<commit_message>
# Day 37 Added
</commit_message>
<xml_diff>
--- a/12620514.xlsx
+++ b/12620514.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D9408FD-BEA4-451A-974D-621307C1F64D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA255365-9B78-480D-9037-77179D316F35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="94">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -307,6 +307,9 @@
   <si>
     <t>Today I give CA of Python and solve some DSA type questions for the practice</t>
   </si>
+  <si>
+    <t xml:space="preserve">Attended mentor meeting and and enery level was queit low in in morning but letter in the afternoon I felt energetic </t>
+  </si>
 </sst>
 </file>
 
@@ -483,9 +486,6 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -501,311 +501,14 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="28">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-        <name val="Arial"/>
-        <charset val="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1385,74 +1088,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="22" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="17"/>
-      <c r="J1" s="17"/>
-      <c r="K1" s="17"/>
-      <c r="L1" s="17"/>
-      <c r="M1" s="17"/>
-      <c r="N1" s="17"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22"/>
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="18" t="s">
+      <c r="B2" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
       <c r="E2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="23">
         <v>12620514</v>
       </c>
-      <c r="G2" s="18"/>
+      <c r="G2" s="23"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="18" t="s">
+      <c r="B3" s="23" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="18"/>
-      <c r="D3" s="18"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="18" t="s">
+      <c r="F3" s="23" t="s">
         <v>37</v>
       </c>
-      <c r="G3" s="18"/>
+      <c r="G3" s="23"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="16" t="s">
+      <c r="A4" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="B4" s="16"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
     </row>
     <row r="5" spans="1:14" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -1545,600 +1248,600 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="19">
+      <c r="A7" s="16">
         <v>46251</v>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="17">
         <v>480</v>
       </c>
-      <c r="C7" s="20">
+      <c r="C7" s="17">
         <v>0</v>
       </c>
-      <c r="D7" s="20">
+      <c r="D7" s="17">
         <v>360</v>
       </c>
-      <c r="E7" s="20">
+      <c r="E7" s="17">
         <v>60</v>
       </c>
-      <c r="F7" s="20">
+      <c r="F7" s="17">
         <v>0</v>
       </c>
-      <c r="G7" s="20">
+      <c r="G7" s="17">
         <v>0</v>
       </c>
-      <c r="H7" s="20">
+      <c r="H7" s="17">
         <v>120</v>
       </c>
-      <c r="I7" s="21">
+      <c r="I7" s="18">
         <f t="shared" si="0"/>
         <v>1020</v>
       </c>
-      <c r="J7" s="21">
+      <c r="J7" s="18">
         <f t="shared" si="1"/>
         <v>420</v>
       </c>
-      <c r="K7" s="22" t="s">
+      <c r="K7" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L7" s="22" t="s">
+      <c r="L7" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N7" s="23" t="s">
+      <c r="N7" s="20" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="19">
+      <c r="A8" s="16">
         <v>46252</v>
       </c>
-      <c r="B8" s="20">
+      <c r="B8" s="17">
         <v>420</v>
       </c>
-      <c r="C8" s="20">
+      <c r="C8" s="17">
         <v>0</v>
       </c>
-      <c r="D8" s="20">
+      <c r="D8" s="17">
         <v>240</v>
       </c>
-      <c r="E8" s="20">
+      <c r="E8" s="17">
         <v>45</v>
       </c>
-      <c r="F8" s="20">
+      <c r="F8" s="17">
         <v>300</v>
       </c>
-      <c r="G8" s="20">
+      <c r="G8" s="17">
         <v>3</v>
       </c>
-      <c r="H8" s="20">
+      <c r="H8" s="17">
         <v>240</v>
       </c>
-      <c r="I8" s="21">
+      <c r="I8" s="18">
         <f t="shared" si="0"/>
         <v>1245</v>
       </c>
-      <c r="J8" s="21">
+      <c r="J8" s="18">
         <f t="shared" si="1"/>
         <v>195</v>
       </c>
-      <c r="K8" s="22" t="s">
+      <c r="K8" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L8" s="22" t="s">
+      <c r="L8" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M8" s="22" t="s">
+      <c r="M8" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="N8" s="23" t="s">
+      <c r="N8" s="20" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="19">
+      <c r="A9" s="16">
         <v>46253</v>
       </c>
-      <c r="B9" s="20">
+      <c r="B9" s="17">
         <v>480</v>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="17">
         <v>0</v>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="17">
         <v>0</v>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="17">
         <v>0</v>
       </c>
-      <c r="F9" s="20">
+      <c r="F9" s="17">
         <v>420</v>
       </c>
-      <c r="G9" s="20">
+      <c r="G9" s="17">
         <v>3</v>
       </c>
-      <c r="H9" s="20">
+      <c r="H9" s="17">
         <v>300</v>
       </c>
-      <c r="I9" s="21">
+      <c r="I9" s="18">
         <f t="shared" si="0"/>
         <v>1200</v>
       </c>
-      <c r="J9" s="21">
+      <c r="J9" s="18">
         <f t="shared" si="1"/>
         <v>240</v>
       </c>
-      <c r="K9" s="22" t="s">
+      <c r="K9" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="L9" s="22" t="s">
+      <c r="L9" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="M9" s="22" t="s">
+      <c r="M9" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="N9" s="23" t="s">
+      <c r="N9" s="20" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="19">
+      <c r="A10" s="16">
         <v>46254</v>
       </c>
-      <c r="B10" s="20">
+      <c r="B10" s="17">
         <v>400</v>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="17">
         <v>0</v>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="17">
         <v>180</v>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="17">
         <v>0</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="17">
         <v>360</v>
       </c>
-      <c r="G10" s="20">
+      <c r="G10" s="17">
         <v>6</v>
       </c>
-      <c r="H10" s="20">
+      <c r="H10" s="17">
         <v>250</v>
       </c>
-      <c r="I10" s="21">
+      <c r="I10" s="18">
         <f t="shared" si="0"/>
         <v>1190</v>
       </c>
-      <c r="J10" s="21">
+      <c r="J10" s="18">
         <f t="shared" si="1"/>
         <v>250</v>
       </c>
-      <c r="K10" s="22" t="s">
+      <c r="K10" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L10" s="22" t="s">
+      <c r="L10" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M10" s="22" t="s">
+      <c r="M10" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N10" s="23" t="s">
+      <c r="N10" s="20" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="19">
+      <c r="A11" s="16">
         <v>46255</v>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="17">
         <v>450</v>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="17">
         <v>20</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="17">
         <v>240</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="17">
         <v>30</v>
       </c>
-      <c r="F11" s="20">
+      <c r="F11" s="17">
         <v>360</v>
       </c>
-      <c r="G11" s="20">
+      <c r="G11" s="17">
         <v>6</v>
       </c>
-      <c r="H11" s="20">
+      <c r="H11" s="17">
         <v>200</v>
       </c>
-      <c r="I11" s="21">
+      <c r="I11" s="18">
         <f t="shared" si="0"/>
         <v>1300</v>
       </c>
-      <c r="J11" s="21">
+      <c r="J11" s="18">
         <f t="shared" si="1"/>
         <v>140</v>
       </c>
-      <c r="K11" s="22" t="s">
+      <c r="K11" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L11" s="22" t="s">
+      <c r="L11" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M11" s="22" t="s">
+      <c r="M11" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N11" s="23" t="s">
+      <c r="N11" s="20" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A12" s="19">
+      <c r="A12" s="16">
         <v>46256</v>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="17">
         <v>540</v>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="17">
         <v>0</v>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="17">
         <v>450</v>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="17">
         <v>120</v>
       </c>
-      <c r="F12" s="20">
+      <c r="F12" s="17">
         <v>0</v>
       </c>
-      <c r="G12" s="20">
+      <c r="G12" s="17">
         <v>0</v>
       </c>
-      <c r="H12" s="20">
+      <c r="H12" s="17">
         <v>300</v>
       </c>
-      <c r="I12" s="21">
+      <c r="I12" s="18">
         <f t="shared" si="0"/>
         <v>1410</v>
       </c>
-      <c r="J12" s="21">
+      <c r="J12" s="18">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="K12" s="22" t="s">
+      <c r="K12" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L12" s="22" t="s">
+      <c r="L12" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M12" s="22" t="s">
+      <c r="M12" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N12" s="23" t="s">
+      <c r="N12" s="20" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="19">
+      <c r="A13" s="16">
         <v>46257</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="17">
         <v>420</v>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="17">
         <v>30</v>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="17">
         <v>390</v>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="17">
         <v>150</v>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="17">
         <v>0</v>
       </c>
-      <c r="G13" s="20">
+      <c r="G13" s="17">
         <v>0</v>
       </c>
-      <c r="H13" s="20">
+      <c r="H13" s="17">
         <v>350</v>
       </c>
-      <c r="I13" s="21">
+      <c r="I13" s="18">
         <f t="shared" si="0"/>
         <v>1340</v>
       </c>
-      <c r="J13" s="21">
+      <c r="J13" s="18">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="K13" s="22" t="s">
+      <c r="K13" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L13" s="22" t="s">
+      <c r="L13" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M13" s="22" t="s">
+      <c r="M13" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N13" s="23" t="s">
+      <c r="N13" s="20" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="19">
+      <c r="A14" s="16">
         <v>46258</v>
       </c>
-      <c r="B14" s="20">
+      <c r="B14" s="17">
         <v>390</v>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="17">
         <v>0</v>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="17">
         <v>480</v>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="17">
         <v>150</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="17">
         <v>240</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="17">
         <v>4</v>
       </c>
-      <c r="H14" s="20">
+      <c r="H14" s="17">
         <v>180</v>
       </c>
-      <c r="I14" s="21">
+      <c r="I14" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J14" s="21">
+      <c r="J14" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K14" s="22" t="s">
+      <c r="K14" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="L14" s="22" t="s">
+      <c r="L14" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="M14" s="22" t="s">
+      <c r="M14" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="N14" s="23" t="s">
+      <c r="N14" s="20" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="19">
+      <c r="A15" s="16">
         <v>46259</v>
       </c>
-      <c r="B15" s="20">
+      <c r="B15" s="17">
         <v>420</v>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="17">
         <v>20</v>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="17">
         <v>450</v>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="17">
         <v>70</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="17">
         <v>360</v>
       </c>
-      <c r="G15" s="20">
+      <c r="G15" s="17">
         <v>6</v>
       </c>
-      <c r="H15" s="20">
+      <c r="H15" s="17">
         <v>100</v>
       </c>
-      <c r="I15" s="21">
+      <c r="I15" s="18">
         <f t="shared" si="0"/>
         <v>1420</v>
       </c>
-      <c r="J15" s="21">
+      <c r="J15" s="18">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="K15" s="22" t="s">
+      <c r="K15" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L15" s="22" t="s">
+      <c r="L15" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M15" s="22" t="s">
+      <c r="M15" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N15" s="23" t="s">
+      <c r="N15" s="20" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A16" s="19">
+      <c r="A16" s="16">
         <v>46260</v>
       </c>
-      <c r="B16" s="20">
+      <c r="B16" s="17">
         <v>420</v>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="17">
         <v>30</v>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="17">
         <v>400</v>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="17">
         <v>100</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="17">
         <v>360</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="17">
         <v>6</v>
       </c>
-      <c r="H16" s="20">
+      <c r="H16" s="17">
         <v>100</v>
       </c>
-      <c r="I16" s="21">
+      <c r="I16" s="18">
         <f t="shared" si="0"/>
         <v>1410</v>
       </c>
-      <c r="J16" s="21">
+      <c r="J16" s="18">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="K16" s="22" t="s">
+      <c r="K16" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L16" s="22" t="s">
+      <c r="L16" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M16" s="22" t="s">
+      <c r="M16" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N16" s="23" t="s">
+      <c r="N16" s="20" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="19">
+      <c r="A17" s="16">
         <v>46261</v>
       </c>
-      <c r="B17" s="20">
+      <c r="B17" s="17">
         <v>300</v>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="17">
         <v>30</v>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="17">
         <v>300</v>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="17">
         <v>120</v>
       </c>
-      <c r="F17" s="20">
+      <c r="F17" s="17">
         <v>360</v>
       </c>
-      <c r="G17" s="20">
+      <c r="G17" s="17">
         <v>6</v>
       </c>
-      <c r="H17" s="20">
+      <c r="H17" s="17">
         <v>300</v>
       </c>
-      <c r="I17" s="21">
+      <c r="I17" s="18">
         <f t="shared" si="0"/>
         <v>1410</v>
       </c>
-      <c r="J17" s="21">
+      <c r="J17" s="18">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="K17" s="22" t="s">
+      <c r="K17" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="L17" s="22" t="s">
+      <c r="L17" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M17" s="22" t="s">
+      <c r="M17" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N17" s="23" t="s">
+      <c r="N17" s="20" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="19">
+      <c r="A18" s="16">
         <v>46262</v>
       </c>
-      <c r="B18" s="20">
+      <c r="B18" s="17">
         <v>420</v>
       </c>
-      <c r="C18" s="20">
+      <c r="C18" s="17">
         <v>0</v>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="17">
         <v>250</v>
       </c>
-      <c r="E18" s="20">
+      <c r="E18" s="17">
         <v>60</v>
       </c>
-      <c r="F18" s="20">
+      <c r="F18" s="17">
         <v>420</v>
       </c>
-      <c r="G18" s="20">
+      <c r="G18" s="17">
         <v>7</v>
       </c>
-      <c r="H18" s="20">
+      <c r="H18" s="17">
         <v>250</v>
       </c>
-      <c r="I18" s="21">
+      <c r="I18" s="18">
         <f t="shared" si="0"/>
         <v>1400</v>
       </c>
-      <c r="J18" s="21">
+      <c r="J18" s="18">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="K18" s="22" t="s">
+      <c r="K18" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L18" s="22" t="s">
+      <c r="L18" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M18" s="22" t="s">
+      <c r="M18" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="N18" s="23" t="s">
+      <c r="N18" s="20" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A19" s="19">
+      <c r="A19" s="16">
         <v>46263</v>
       </c>
-      <c r="B19" s="20">
+      <c r="B19" s="17">
         <v>300</v>
       </c>
-      <c r="C19" s="20">
+      <c r="C19" s="17">
         <v>0</v>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="17">
         <v>200</v>
       </c>
-      <c r="E19" s="20">
+      <c r="E19" s="17">
         <v>0</v>
       </c>
-      <c r="F19" s="20">
+      <c r="F19" s="17">
         <v>0</v>
       </c>
-      <c r="G19" s="20">
+      <c r="G19" s="17">
         <v>0</v>
       </c>
-      <c r="H19" s="20">
+      <c r="H19" s="17">
         <v>900</v>
       </c>
-      <c r="I19" s="21">
+      <c r="I19" s="18">
         <f t="shared" si="0"/>
         <v>1400</v>
       </c>
-      <c r="J19" s="21">
+      <c r="J19" s="18">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="K19" s="22" t="s">
+      <c r="K19" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="L19" s="22" t="s">
+      <c r="L19" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="M19" s="22" t="s">
+      <c r="M19" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="N19" s="23" t="s">
+      <c r="N19" s="20" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2189,646 +1892,646 @@
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A21" s="19">
+      <c r="A21" s="16">
         <v>46265</v>
       </c>
-      <c r="B21" s="20">
+      <c r="B21" s="17">
         <v>420</v>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="17">
         <v>0</v>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="17">
         <v>450</v>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="17">
         <v>120</v>
       </c>
-      <c r="F21" s="20">
+      <c r="F21" s="17">
         <v>120</v>
       </c>
-      <c r="G21" s="20">
+      <c r="G21" s="17">
         <v>2</v>
       </c>
-      <c r="H21" s="20">
+      <c r="H21" s="17">
         <v>300</v>
       </c>
-      <c r="I21" s="21">
+      <c r="I21" s="18">
         <f t="shared" si="0"/>
         <v>1410</v>
       </c>
-      <c r="J21" s="21">
+      <c r="J21" s="18">
         <f t="shared" si="1"/>
         <v>30</v>
       </c>
-      <c r="K21" s="22" t="s">
+      <c r="K21" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L21" s="22" t="s">
+      <c r="L21" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M21" s="22" t="s">
+      <c r="M21" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N21" s="23" t="s">
+      <c r="N21" s="20" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A22" s="19">
+      <c r="A22" s="16">
         <v>46266</v>
       </c>
-      <c r="B22" s="20">
+      <c r="B22" s="17">
         <v>360</v>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="17">
         <v>30</v>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="17">
         <v>180</v>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="17">
         <v>30</v>
       </c>
-      <c r="F22" s="20">
+      <c r="F22" s="17">
         <v>360</v>
       </c>
-      <c r="G22" s="20">
+      <c r="G22" s="17">
         <v>5</v>
       </c>
-      <c r="H22" s="20">
+      <c r="H22" s="17">
         <v>480</v>
       </c>
-      <c r="I22" s="21">
+      <c r="I22" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J22" s="21">
+      <c r="J22" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K22" s="22" t="s">
+      <c r="K22" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L22" s="22" t="s">
+      <c r="L22" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M22" s="22" t="s">
+      <c r="M22" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N22" s="23" t="s">
+      <c r="N22" s="20" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A23" s="19">
+      <c r="A23" s="16">
         <v>46267</v>
       </c>
-      <c r="B23" s="20">
+      <c r="B23" s="17">
         <v>360</v>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="17">
         <v>0</v>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="17">
         <v>200</v>
       </c>
-      <c r="E23" s="20">
+      <c r="E23" s="17">
         <v>60</v>
       </c>
-      <c r="F23" s="20">
+      <c r="F23" s="17">
         <v>360</v>
       </c>
-      <c r="G23" s="20">
+      <c r="G23" s="17">
         <v>5</v>
       </c>
-      <c r="H23" s="20">
+      <c r="H23" s="17">
         <v>460</v>
       </c>
-      <c r="I23" s="21">
+      <c r="I23" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J23" s="21">
+      <c r="J23" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K23" s="22" t="s">
+      <c r="K23" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L23" s="22" t="s">
+      <c r="L23" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M23" s="22" t="s">
+      <c r="M23" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="N23" s="23" t="s">
+      <c r="N23" s="20" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A24" s="19">
+      <c r="A24" s="16">
         <v>46268</v>
       </c>
-      <c r="B24" s="20">
+      <c r="B24" s="17">
         <v>327</v>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="17">
         <v>0</v>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="17">
         <v>300</v>
       </c>
-      <c r="E24" s="20">
+      <c r="E24" s="17">
         <v>60</v>
       </c>
-      <c r="F24" s="20">
+      <c r="F24" s="17">
         <v>360</v>
       </c>
-      <c r="G24" s="20">
+      <c r="G24" s="17">
         <v>6</v>
       </c>
-      <c r="H24" s="20">
+      <c r="H24" s="17">
         <v>390</v>
       </c>
-      <c r="I24" s="21">
+      <c r="I24" s="18">
         <f t="shared" si="0"/>
         <v>1437</v>
       </c>
-      <c r="J24" s="21">
+      <c r="J24" s="18">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="K24" s="22" t="s">
+      <c r="K24" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L24" s="22" t="s">
+      <c r="L24" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M24" s="22" t="s">
+      <c r="M24" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N24" s="23" t="s">
+      <c r="N24" s="20" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A25" s="19">
+      <c r="A25" s="16">
         <v>46269</v>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="17">
         <v>387</v>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="17">
         <v>0</v>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="17">
         <v>300</v>
       </c>
-      <c r="E25" s="20">
+      <c r="E25" s="17">
         <v>120</v>
       </c>
-      <c r="F25" s="20">
+      <c r="F25" s="17">
         <v>420</v>
       </c>
-      <c r="G25" s="20">
+      <c r="G25" s="17">
         <v>7</v>
       </c>
-      <c r="H25" s="20">
+      <c r="H25" s="17">
         <v>200</v>
       </c>
-      <c r="I25" s="21">
+      <c r="I25" s="18">
         <f t="shared" si="0"/>
         <v>1427</v>
       </c>
-      <c r="J25" s="21">
+      <c r="J25" s="18">
         <f t="shared" si="1"/>
         <v>13</v>
       </c>
-      <c r="K25" s="22" t="s">
+      <c r="K25" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L25" s="22" t="s">
+      <c r="L25" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M25" s="22" t="s">
+      <c r="M25" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N25" s="23" t="s">
+      <c r="N25" s="20" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="19">
+      <c r="A26" s="16">
         <v>46270</v>
       </c>
-      <c r="B26" s="20">
+      <c r="B26" s="17">
         <v>300</v>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="17">
         <v>20</v>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="17">
         <v>360</v>
       </c>
-      <c r="E26" s="20">
+      <c r="E26" s="17">
         <v>60</v>
       </c>
-      <c r="F26" s="20">
+      <c r="F26" s="17">
         <v>240</v>
       </c>
-      <c r="G26" s="20">
+      <c r="G26" s="17">
         <v>4</v>
       </c>
-      <c r="H26" s="20">
+      <c r="H26" s="17">
         <v>460</v>
       </c>
-      <c r="I26" s="21">
+      <c r="I26" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J26" s="21">
+      <c r="J26" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K26" s="22" t="s">
+      <c r="K26" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L26" s="22" t="s">
+      <c r="L26" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M26" s="22" t="s">
+      <c r="M26" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N26" s="23" t="s">
+      <c r="N26" s="20" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A27" s="19">
+      <c r="A27" s="16">
         <v>46271</v>
       </c>
-      <c r="B27" s="20">
+      <c r="B27" s="17">
         <v>320</v>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="17">
         <v>50</v>
       </c>
-      <c r="D27" s="20">
+      <c r="D27" s="17">
         <v>360</v>
       </c>
-      <c r="E27" s="20">
+      <c r="E27" s="17">
         <v>120</v>
       </c>
-      <c r="F27" s="20">
+      <c r="F27" s="17">
         <v>300</v>
       </c>
-      <c r="G27" s="20">
+      <c r="G27" s="17">
         <v>5</v>
       </c>
-      <c r="H27" s="20">
+      <c r="H27" s="17">
         <v>290</v>
       </c>
-      <c r="I27" s="21">
+      <c r="I27" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J27" s="21">
+      <c r="J27" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K27" s="22" t="s">
+      <c r="K27" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L27" s="22" t="s">
+      <c r="L27" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="M27" s="22" t="s">
+      <c r="M27" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N27" s="23" t="s">
+      <c r="N27" s="20" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="19">
+      <c r="A28" s="16">
         <v>46272</v>
       </c>
-      <c r="B28" s="20">
+      <c r="B28" s="17">
         <v>180</v>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="17">
         <v>30</v>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="17">
         <v>420</v>
       </c>
-      <c r="E28" s="20">
+      <c r="E28" s="17">
         <v>120</v>
       </c>
-      <c r="F28" s="20">
+      <c r="F28" s="17">
         <v>360</v>
       </c>
-      <c r="G28" s="20">
+      <c r="G28" s="17">
         <v>6</v>
       </c>
-      <c r="H28" s="20">
+      <c r="H28" s="17">
         <v>330</v>
       </c>
-      <c r="I28" s="21">
+      <c r="I28" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J28" s="21">
+      <c r="J28" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K28" s="22" t="s">
+      <c r="K28" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L28" s="22" t="s">
+      <c r="L28" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M28" s="22" t="s">
+      <c r="M28" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N28" s="23" t="s">
+      <c r="N28" s="20" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="19">
+      <c r="A29" s="16">
         <v>46273</v>
       </c>
-      <c r="B29" s="20">
+      <c r="B29" s="17">
         <v>240</v>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="17">
         <v>60</v>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="17">
         <v>360</v>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="17">
         <v>125</v>
       </c>
-      <c r="F29" s="20">
+      <c r="F29" s="17">
         <v>360</v>
       </c>
-      <c r="G29" s="20">
+      <c r="G29" s="17">
         <v>6</v>
       </c>
-      <c r="H29" s="20">
+      <c r="H29" s="17">
         <v>295</v>
       </c>
-      <c r="I29" s="21">
+      <c r="I29" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J29" s="21">
+      <c r="J29" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K29" s="22" t="s">
+      <c r="K29" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L29" s="22" t="s">
+      <c r="L29" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M29" s="22" t="s">
+      <c r="M29" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N29" s="23" t="s">
+      <c r="N29" s="20" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A30" s="19">
+      <c r="A30" s="16">
         <v>46274</v>
       </c>
-      <c r="B30" s="20">
+      <c r="B30" s="17">
         <v>180</v>
       </c>
-      <c r="C30" s="20">
+      <c r="C30" s="17">
         <v>30</v>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="17">
         <v>480</v>
       </c>
-      <c r="E30" s="20">
+      <c r="E30" s="17">
         <v>150</v>
       </c>
-      <c r="F30" s="20">
+      <c r="F30" s="17">
         <v>360</v>
       </c>
-      <c r="G30" s="20">
+      <c r="G30" s="17">
         <v>6</v>
       </c>
-      <c r="H30" s="20">
+      <c r="H30" s="17">
         <v>240</v>
       </c>
-      <c r="I30" s="21">
+      <c r="I30" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J30" s="21">
+      <c r="J30" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K30" s="22" t="s">
+      <c r="K30" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L30" s="22" t="s">
+      <c r="L30" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M30" s="22" t="s">
+      <c r="M30" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N30" s="23" t="s">
+      <c r="N30" s="20" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A31" s="19">
+      <c r="A31" s="16">
         <v>46275</v>
       </c>
-      <c r="B31" s="20">
+      <c r="B31" s="17">
         <v>240</v>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="17">
         <v>0</v>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="17">
         <v>420</v>
       </c>
-      <c r="E31" s="20">
+      <c r="E31" s="17">
         <v>120</v>
       </c>
-      <c r="F31" s="20">
+      <c r="F31" s="17">
         <v>360</v>
       </c>
-      <c r="G31" s="20">
+      <c r="G31" s="17">
         <v>6</v>
       </c>
-      <c r="H31" s="20">
+      <c r="H31" s="17">
         <v>300</v>
       </c>
-      <c r="I31" s="21">
+      <c r="I31" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J31" s="21">
+      <c r="J31" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K31" s="22" t="s">
+      <c r="K31" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L31" s="22" t="s">
+      <c r="L31" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M31" s="22" t="s">
+      <c r="M31" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="N31" s="23" t="s">
+      <c r="N31" s="20" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A32" s="19">
+      <c r="A32" s="16">
         <v>46276</v>
       </c>
-      <c r="B32" s="20">
+      <c r="B32" s="17">
         <v>300</v>
       </c>
-      <c r="C32" s="20">
+      <c r="C32" s="17">
         <v>0</v>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="17">
         <v>120</v>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="17">
         <v>0</v>
       </c>
-      <c r="F32" s="20">
+      <c r="F32" s="17">
         <v>420</v>
       </c>
-      <c r="G32" s="20">
+      <c r="G32" s="17">
         <v>7</v>
       </c>
-      <c r="H32" s="20">
+      <c r="H32" s="17">
         <v>600</v>
       </c>
-      <c r="I32" s="21">
+      <c r="I32" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J32" s="21">
+      <c r="J32" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K32" s="22" t="s">
+      <c r="K32" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L32" s="22" t="s">
+      <c r="L32" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M32" s="22" t="s">
+      <c r="M32" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N32" s="23" t="s">
+      <c r="N32" s="20" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="19">
+      <c r="A33" s="16">
         <v>46277</v>
       </c>
-      <c r="B33" s="20">
+      <c r="B33" s="17">
         <v>480</v>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="17">
         <v>0</v>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="17">
         <v>500</v>
       </c>
-      <c r="E33" s="20">
+      <c r="E33" s="17">
         <v>60</v>
       </c>
-      <c r="F33" s="20">
+      <c r="F33" s="17">
         <v>0</v>
       </c>
-      <c r="G33" s="20">
+      <c r="G33" s="17">
         <v>0</v>
       </c>
-      <c r="H33" s="20">
+      <c r="H33" s="17">
         <v>400</v>
       </c>
-      <c r="I33" s="21">
+      <c r="I33" s="18">
         <f t="shared" si="0"/>
         <v>1440</v>
       </c>
-      <c r="J33" s="21">
+      <c r="J33" s="18">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K33" s="22" t="s">
+      <c r="K33" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L33" s="22" t="s">
+      <c r="L33" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M33" s="22" t="s">
+      <c r="M33" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N33" s="23" t="s">
+      <c r="N33" s="20" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A34" s="19">
+      <c r="A34" s="16">
         <v>46278</v>
       </c>
-      <c r="B34" s="20">
+      <c r="B34" s="17">
         <v>480</v>
       </c>
-      <c r="C34" s="20">
+      <c r="C34" s="17">
         <v>30</v>
       </c>
-      <c r="D34" s="20">
+      <c r="D34" s="17">
         <v>300</v>
       </c>
-      <c r="E34" s="20">
+      <c r="E34" s="17">
         <v>30</v>
       </c>
-      <c r="F34" s="20">
+      <c r="F34" s="17">
         <v>0</v>
       </c>
-      <c r="G34" s="20">
+      <c r="G34" s="17">
         <v>0</v>
       </c>
-      <c r="H34" s="20">
+      <c r="H34" s="17">
         <v>500</v>
       </c>
-      <c r="I34" s="21">
+      <c r="I34" s="18">
         <f t="shared" si="0"/>
         <v>1340</v>
       </c>
-      <c r="J34" s="21">
+      <c r="J34" s="18">
         <f t="shared" si="1"/>
         <v>100</v>
       </c>
-      <c r="K34" s="22" t="s">
+      <c r="K34" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="L34" s="22" t="s">
+      <c r="L34" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="M34" s="22" t="s">
+      <c r="M34" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="N34" s="23" t="s">
+      <c r="N34" s="20" t="s">
         <v>91</v>
       </c>
     </row>
@@ -2877,72 +2580,97 @@
       </c>
     </row>
     <row r="36" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="19">
+      <c r="A36" s="16">
         <v>46280</v>
       </c>
-      <c r="B36" s="20">
+      <c r="B36" s="17">
         <v>300</v>
       </c>
-      <c r="C36" s="20">
+      <c r="C36" s="17">
         <v>50</v>
       </c>
-      <c r="D36" s="20">
+      <c r="D36" s="17">
         <v>120</v>
       </c>
-      <c r="E36" s="20">
+      <c r="E36" s="17">
         <v>60</v>
       </c>
-      <c r="F36" s="20">
+      <c r="F36" s="17">
         <v>300</v>
       </c>
-      <c r="G36" s="20">
+      <c r="G36" s="17">
         <v>5</v>
       </c>
-      <c r="H36" s="20">
+      <c r="H36" s="17">
         <v>510</v>
       </c>
-      <c r="I36" s="21">
+      <c r="I36" s="18">
         <f>IF(SUM(B36:F36,H36)=0,"",SUM(B36:F36,H36))</f>
         <v>1340</v>
       </c>
-      <c r="J36" s="21">
+      <c r="J36" s="18">
         <f t="shared" ref="J36" si="2">IF(I36="","",1440-I36)</f>
         <v>100</v>
       </c>
-      <c r="K36" s="22" t="s">
+      <c r="K36" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="L36" s="22" t="s">
+      <c r="L36" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="M36" s="22" t="s">
+      <c r="M36" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="N36" s="23" t="s">
+      <c r="N36" s="20" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="12"/>
-      <c r="B37" s="13"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="13"/>
-      <c r="G37" s="13"/>
-      <c r="H37" s="13"/>
-      <c r="I37" s="14" t="str">
+    <row r="37" spans="1:14" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="A37" s="12">
+        <v>46281</v>
+      </c>
+      <c r="B37" s="13">
+        <v>360</v>
+      </c>
+      <c r="C37" s="13">
+        <v>0</v>
+      </c>
+      <c r="D37" s="13">
+        <v>180</v>
+      </c>
+      <c r="E37" s="13">
+        <v>60</v>
+      </c>
+      <c r="F37" s="13">
+        <f>60*3</f>
+        <v>180</v>
+      </c>
+      <c r="G37" s="13">
+        <v>3</v>
+      </c>
+      <c r="H37" s="13">
+        <v>500</v>
+      </c>
+      <c r="I37" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="14" t="str">
+        <v>1280</v>
+      </c>
+      <c r="J37" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="13"/>
-      <c r="L37" s="13"/>
-      <c r="M37" s="13"/>
-      <c r="N37" s="15"/>
+        <v>160</v>
+      </c>
+      <c r="K37" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="L37" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="M37" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="N37" s="15" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A38" s="12"/>
@@ -11247,137 +10975,12 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J7">
-    <cfRule type="cellIs" dxfId="27" priority="28" operator="lessThan">
+  <conditionalFormatting sqref="J7:J19">
+    <cfRule type="cellIs" dxfId="2" priority="16" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J8">
-    <cfRule type="cellIs" dxfId="26" priority="27" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J9">
-    <cfRule type="cellIs" dxfId="25" priority="26" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J10">
-    <cfRule type="cellIs" dxfId="24" priority="25" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
-    <cfRule type="cellIs" dxfId="23" priority="24" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J12">
-    <cfRule type="cellIs" dxfId="22" priority="23" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J13">
-    <cfRule type="cellIs" dxfId="21" priority="22" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J14">
-    <cfRule type="cellIs" dxfId="20" priority="21" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J15">
-    <cfRule type="cellIs" dxfId="19" priority="20" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J16">
-    <cfRule type="cellIs" dxfId="18" priority="19" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J17">
-    <cfRule type="cellIs" dxfId="17" priority="18" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J18">
-    <cfRule type="cellIs" dxfId="16" priority="17" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J19">
-    <cfRule type="cellIs" dxfId="15" priority="16" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J21">
-    <cfRule type="cellIs" dxfId="14" priority="15" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J22">
-    <cfRule type="cellIs" dxfId="13" priority="14" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J23">
-    <cfRule type="cellIs" dxfId="12" priority="13" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J24">
-    <cfRule type="cellIs" dxfId="11" priority="12" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J25">
-    <cfRule type="cellIs" dxfId="10" priority="11" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J26">
-    <cfRule type="cellIs" dxfId="9" priority="10" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J27">
-    <cfRule type="cellIs" dxfId="8" priority="9" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J28">
-    <cfRule type="cellIs" dxfId="7" priority="8" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J29">
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J30">
-    <cfRule type="cellIs" dxfId="5" priority="6" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J31">
-    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J32">
-    <cfRule type="cellIs" dxfId="3" priority="4" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J33">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J34">
+  <conditionalFormatting sqref="J21:J34">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
       <formula>0</formula>
     </cfRule>

</xml_diff>